<commit_message>
layout: light theme + content-driven design + section-based data filter
主题与布局：
- 浅色专业风（白底 + 浅边框 + 微妙阴影，参考企业仪表盘）
- 按 .docx 内容比重定制每个模块排版：
  - M-1 组织架构：1 full-width hierarchy（隐藏次要 ranking）
  - M-2 员工情况：3 compact KPIs + 4 half sections（age/edu/gender/customer）
  - M-3 人员优化：3 compact KPIs + funnel half + progress half + 1 full
  - M-4 干部队伍：3 compact KPIs + table full + ranking full
  - M-5 考核薪酬：4 compact KPIs + 1 full ranking
  - M-6 培训赋能：3 compact KPIs + 2 full (progress + ranking)

数据切片机制：
- test data 加 'section' 列，每行声明归属
- composer _adapt_and_render 按 data_key 过滤 rows
- 修复 bar.py 字符串 value 崩 f-string
- progress viz 自动从 sub 字段提取 target 数

size: 44422 bytes (43.4KB, ≤ 50KB)
</commit_message>
<xml_diff>
--- a/data/test.xlsx
+++ b/data/test.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>人力资源管理数据驾驶舱（测试）</t>
+          <t>人力资源管理数据驾驶舱</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>#1E5BAA</t>
+          <t>#1e5baa</t>
         </is>
       </c>
     </row>
@@ -493,46 +493,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>区域</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>机构</t>
+          <t>region</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>广州</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>广州分行</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>37</v>
-      </c>
-      <c r="D2" t="inlineStr">
+          <t>总行本部</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>一级部门</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>28</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -541,18 +551,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>广州</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>海珠支行</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>22</v>
-      </c>
-      <c r="D3" t="inlineStr">
+          <t>总行本部</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>二级部门</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>13</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -561,18 +576,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>广州</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>天河支行</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D4" t="inlineStr">
+          <t>总行直属</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>一级部门</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -581,18 +601,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>异地</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>深圳分行</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="inlineStr">
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>广州分行</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>37</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -601,18 +626,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>异地</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>佛山分行</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="inlineStr">
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>海珠中心支行</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -621,18 +651,423 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>异地</t>
+          <t>region_tree</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>天河中心支行</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>白云中心支行</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>开发区中心支行</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>增城中心支行</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>南沙分行</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>科技支行</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>广州地区</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>行总营业部</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>深圳分行</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>佛山分行</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>南京分行</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="D16" t="n">
         <v>9</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>惠州分行</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>江门分行</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>中山分行</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>肇庆分行</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>东莞分行</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>横琴分行</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>营业</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>region_tree</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>异地地区</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>清远分行</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>营业</t>
         </is>
@@ -649,282 +1084,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>维度</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>类别</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>占比</t>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>headcount_total</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30岁以下</t>
+          <t>正式员工</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1526</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.2586</v>
+        <v>5901</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>含劳务派遣 6589</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>headcount_operating</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>31-40岁</t>
+          <t>经营机构</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2851</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.4831</v>
+        <v>4709</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>占 79.80%</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>headcount_ratio</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41-50岁</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1123</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.1903</v>
+          <t>前中后台</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1:0.73</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>前 3254 : 中后台 2372</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>年龄</t>
+          <t>age_distribution</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>51岁以上</t>
+          <t>30岁以下</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>401</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.068</v>
-      </c>
+        <v>1526</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>学历</t>
+          <t>age_distribution</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>硕士及以上</t>
+          <t>31-40岁</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1031</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.1747</v>
-      </c>
+        <v>2851</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>学历</t>
+          <t>age_distribution</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>本科</t>
+          <t>41-50岁</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4514</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.765</v>
-      </c>
+        <v>1123</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>学历</t>
+          <t>age_distribution</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>专科</t>
+          <t>51岁以上</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>326</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.0552</v>
-      </c>
+        <v>401</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>学历</t>
+          <t>edu_distribution</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>专科以下</t>
+          <t>硕士及以上</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.0051</v>
-      </c>
+        <v>1031</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>性别</t>
+          <t>edu_distribution</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>本科</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2717</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.4604</v>
-      </c>
+        <v>4514</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>性别</t>
+          <t>edu_distribution</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>专科</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3184</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.5396</v>
-      </c>
+        <v>326</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>客户经理</t>
+          <t>edu_distribution</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>对公</t>
+          <t>专科以下</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>850</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.5024</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>客户经理</t>
+          <t>gender_distribution</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>个人</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>390</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.2305</v>
-      </c>
+        <v>2717</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>客户经理</t>
+          <t>gender_distribution</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>个贷</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>359</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.2122</v>
-      </c>
+        <v>3184</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>客户经理</t>
+          <t>customer_managers</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>微贷</t>
+          <t>对公客户经理</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>850</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>个人客户经理</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>390</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>个贷客户经理</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>359</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>微贷客户经理</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>93</v>
       </c>
-      <c r="D15" t="n">
-        <v>0.055</v>
-      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -937,125 +1406,225 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>指标</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>计划</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>实际</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>完成率</t>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>腾笼换鸟</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>410</v>
+          <t>social_hire_total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>社招入职</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>201</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.5</v>
+        <v>34</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026 年以来</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>绩差退出</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>96</v>
+          <t>campus_hire_total</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>校招签约</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>44</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.46</v>
+        <v>721</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>已签约/签约中</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>社招入职</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
+          <t>exit_total</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>累计退出</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
+        <v>202</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1-5 月</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>校招签约</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>全年目标</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>659</v>
       </c>
-      <c r="C5" t="n">
-        <v>721</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1.09</v>
-      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>总退出</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>已签约</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>202</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
+        <v>721</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>劳动仲裁</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>管培生</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>15</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>金融科技岗</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>54</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>分行管培生</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>112</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>campus_funnel</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>英才岗</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>469</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>teng_long_huan_yao</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>腾笼换鸟</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>201</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>全年任务 410</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>poor_perf_exit</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>绩差退出</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>44</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>目标 50%（96人）</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1069,141 +1638,296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>分类</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>总职数</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>已配</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>空缺</t>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>中层正职</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>54</v>
+          <t>headcount_total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>中层总职数</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>中层副职</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>157</v>
+          <t>headcount_filled</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>已配备</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>144</v>
-      </c>
-      <c r="D3" t="n">
-        <v>13</v>
+        <v>194</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>总行部门</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>100</v>
+          <t>headcount_vacancy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>空缺</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>93</v>
-      </c>
-      <c r="D4" t="n">
-        <v>7</v>
+        <v>17</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>经营机构</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>111</v>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>市管领导干部</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>101</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>提拔</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>94</v>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>高管人员</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>降免</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>派驻纪检监察组</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>中层正职</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>54</v>
+      </c>
+      <c r="D8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>中层副职</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>157</v>
+      </c>
+      <c r="D9" t="n">
+        <v>144</v>
+      </c>
+      <c r="E9" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>总行部门</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" t="n">
+        <v>93</v>
+      </c>
+      <c r="E10" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>config_table</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>经营机构</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>111</v>
+      </c>
+      <c r="D11" t="n">
+        <v>101</v>
+      </c>
+      <c r="E11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>adjustments</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>提拔</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>94</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>adjustments</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>降免职</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>14</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>adjustments</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>到龄转岗</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
+      <c r="C14" t="n">
         <v>13</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1217,128 +1941,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>指标</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025年工资总额</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>15</v>
+          <t>salary_total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025 年工资总额</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>亿元</t>
-        </is>
-      </c>
+          <t>15 亿元</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>salary_per_capita</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>人均薪酬</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>24.3</v>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>万元</t>
+          <t>24.3 万元</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>含预发 2026 开门红 0.3 亿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026年1-5月发放</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4.2</v>
+          <t>pension_balance</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>企业年金余额</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>亿元</t>
+          <t>17.44 亿元</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026.5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>企业年金余额</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>17.44</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>亿元</t>
+          <t>tou_lang_count</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>头狼评选</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>129</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026 Q1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>补充医疗节余</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>亿元</t>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>监测人数</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>95</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>班子成员</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>履职监测黑榜</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>15</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>人次</t>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>监测人次</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>113</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>业绩监测</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>头狼评选</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>129</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>人</t>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>黑榜人数</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>督导函</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>黑榜人次</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>首次触发</t>
         </is>
       </c>
     </row>
@@ -1353,174 +2139,278 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>部门/项目</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>计划</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>完成</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>百分比</t>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>能力大提升</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>983</v>
+          <t>training_total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>能力大提升项目</t>
+        </is>
       </c>
       <c r="C2" t="n">
         <v>983</v>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>key_projects</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>重点培训项目</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>55</v>
       </c>
-      <c r="C3" t="n">
-        <v>32</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.5806</v>
-      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>董事会办公室</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
+          <t>exam_count</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>上岗资格人次</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
+        <v>1878</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>35 场次</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>私人银行部</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
+          <t>key_projects_pct</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>重点项目执行率</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
+        <v>0.5806</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>已完成 32/55</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>金融同业部</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>董事会办公室</t>
+        </is>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>金融科技部</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>私人银行部</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>100</v>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>内控合规部</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>金融同业部</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>100</v>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>运营管理部</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>金融市场部</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>100</v>
       </c>
-      <c r="C9" t="n">
-        <v>14</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.1429</v>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>上岗资格</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>35</v>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>战略客户部</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>1878</v>
-      </c>
-      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>消保部</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>机关纪委</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>安全保卫部</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>金融科技部</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>0</v>
       </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>内控合规部</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dept_execution</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>运营管理部</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
layout: compact dense report (150+ data points, 33.6KB, 3-breakpoint responsive)
新设计目标：
- 信息密度最大化（每行一个数据点）
- 桌面 2-3 列 / 平板 2 列 / 手机 1 列
- 紧凑间距，无大卡片包装
- 全部 .docx 数据点包含

数据流（简化）：
- 每行 [section, label, value, sub]
- composer 按 data_key 过滤 section
- 渲染为 stat-row：label | value | inline-bar | sub
- table 类型：渲染为数据表

响应式断点：
- ≥1100px：auto-fit (min 320px) 多列
- 760-1100px：2 列
- 480-760px：1 列 + 隐藏 sub
- <480px：1 列 + 单列 grid

内容覆盖（vs 原 .docx）：
- M-1 4 sections (总行架构/全行机构/广州网点/异地网点)
- M-2 6 sections (10 员工总数 + age/gender/edu + 客户经理 + 客服)
- M-3 6 sections (社招/校招/退出/腾笼换鸟/绩差/仲裁)
- M-4 3 sections (总览 + 7 行职数表 + 调整)
- M-5 3 sections (薪酬/年金/监测)
- M-6 5 sections (总量/重点/Top/Bottom/考试)
- 共 27 sections / 162 stat-rows / 完整 .docx 数据

size: 34387 bytes (33.6KB, 远低于 50KB)
</commit_message>
<xml_diff>
--- a/data/test.xlsx
+++ b/data/test.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,572 +504,617 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>status</t>
+          <t>sub</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>headquarters</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>总行本部</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>一级部门</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+          <t>总行本部一级部门</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>28</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>营业</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>个</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>headquarters</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>总行本部</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>二级部门</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>13</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>总行直属一级部门</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>个</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>headquarters</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>总行直属</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>一级部门</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>总行直属二级部门</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>个</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branches</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>广州分行</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>37</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>分行级机构</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>家（含总行营业部、信用卡中心）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branches</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>海珠中心支行</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>全行网点</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>183</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branches</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>天河中心支行</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>14</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>正常营业</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>179</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branches</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>白云中心支行</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>12</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>临时停业</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>开发区中心支行</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>11</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>行总营业部</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>增城中心支行</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>广州分行</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>37</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>南沙分行</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>海珠中心支行</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>科技支行</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>天河中心支行</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>广州地区</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>行总营业部</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>白云中心支行</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>深圳分行</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>12</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>开发区中心支行</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>佛山分行</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>12</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>增城中心支行</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>南京分行</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>南沙分行</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_guangzhou</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>惠州分行</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>科技支行</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>江门分行</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>深圳分行</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>中山分行</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>佛山分行</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>肇庆分行</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>南京分行</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>东莞分行</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>惠州分行</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>横琴分行</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>营业</t>
+          <t>江门分行</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>region_tree</t>
+          <t>branch_other</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>异地地区</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+          <t>中山分行</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>肇庆分行</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>东莞分行</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>横琴分行</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>清远分行</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="C27" t="n">
         <v>2</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>营业</t>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>汕头分行</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>韶关分行</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>湛江分行</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>家</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>branch_other</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>梅州分行</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>家</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1112,7 +1157,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>headcount_total</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1125,275 +1170,547 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>含劳务派遣 6589</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>headcount_operating</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>经营机构</t>
+          <t>劳务派遣</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4709</v>
+        <v>688</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>占 79.80%</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>headcount_ratio</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>前中后台</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1:0.73</t>
-        </is>
+          <t>合计总数</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6589</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>前 3254 : 中后台 2372</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>age_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30岁以下</t>
+          <t>总行机关</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1526</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>716</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12.13%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>age_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>31-40岁</t>
+          <t>总行直属机构</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2851</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>476</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8.07%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>age_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>41-50岁</t>
+          <t>经营机构</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1123</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>4709</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>79.80%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>age_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>51岁以上</t>
+          <t>前台</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>401</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>3254</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>edu_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>硕士及以上</t>
+          <t>中后台</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1031</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>2372</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>edu_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>本科</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>4514</v>
+          <t>前中后台比</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1:0.73</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>edu_distribution</t>
+          <t>headcount</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>专科</t>
+          <t>平均年龄</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>326</v>
-      </c>
-      <c r="D11" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>岁</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>edu_distribution</t>
+          <t>age_dist</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>专科以下</t>
+          <t>30岁以下</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>1526</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>25.86%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gender_distribution</t>
+          <t>age_dist</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>31-40岁</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2717</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>2851</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>48.31%</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gender_distribution</t>
+          <t>age_dist</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>41-50岁</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3184</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
+        <v>1123</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>19.03%</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>customer_managers</t>
+          <t>age_dist</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>对公客户经理</t>
+          <t>51岁以上</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>850</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>401</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>customer_managers</t>
+          <t>gender_dist</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>个人客户经理</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>390</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>2717</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>46.04%</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>customer_managers</t>
+          <t>gender_dist</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>个贷客户经理</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>359</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>3184</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>53.96%</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>edu_dist</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>硕士研究生及以上</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>17.47%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>edu_dist</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4514</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>76.50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>edu_dist</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>专科</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>326</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>5.52%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>edu_dist</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>专科以下</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>30</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.51%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>customer_managers</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>客户经理合计</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1692</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>不含 172 劳务派遣</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>对公客户经理</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>850</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>个人客户经理</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>390</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>个贷客户经理</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>359</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>customer_managers</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>微贷客户经理</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C26" t="n">
         <v>93</v>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>service_managers</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>客服经理合计</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1165</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>service_managers</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>客服经理（非临柜）</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>163</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>service_managers</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>客服经理（临柜）</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1002</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1406,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1434,12 +1751,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>social_hire_total</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>社招入职</t>
+          <t>社招合计</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1447,183 +1764,1059 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026 年以来</t>
+          <t>人 · 2026 年以来</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>campus_hire_total</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>校招签约</t>
+          <t>总行总经理助理级以上</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>721</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>已签约/签约中</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>exit_total</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>累计退出</t>
+          <t>分支行部门班子</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>202</v>
+        <v>4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1-5 月</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>全年目标</t>
+          <t>网点班子</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>659</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>已签约</t>
+          <t>各类客户经理</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>721</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>social_hire</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>管培生</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>45</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>campus_hire</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>金融科技岗</t>
+          <t>全年目标</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>659</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>campus_hire</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>分行管培生</t>
+          <t>已签约/签约中</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>112</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>721</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>campus_funnel</t>
+          <t>campus_hire</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>英才岗</t>
+          <t>秋招</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>469</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>250</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>teng_long_huan_yao</t>
+          <t>campus_hire</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>腾笼换鸟</t>
+          <t>春招</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>201</v>
+        <v>430</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>全年任务 410</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>poor_perf_exit</t>
+          <t>campus_hire</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>绩差退出</t>
+          <t>微贷/特资</t>
         </is>
       </c>
       <c r="C12" t="n">
+        <v>41</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>一本及以上占比</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>+7% YoY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>总行管培生</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>总行金融科技岗</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>54</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>分行管培生</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>112</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>英才岗</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>469</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>campus_hire</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>微贷/特资定向</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>41</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>累计退出</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>202</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>人 · 2026 年以来</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>总行直属 离职</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>24</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>总行直属 退休</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>经营机构 离职</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>153</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>经营机构 退休</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>19</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>高管级退休</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>人（胡优华资深督导）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>中层干部 离职</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>员工 离职</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>175</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>员工 退休</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>全年任务</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>410</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1-5月累计退出</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>201</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>任务完成率</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>完成率 Top1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>总营 295%</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>完成率 Top2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>惠州 259%</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>完成率 Top3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>东莞 255%</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>完成量 Top1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>广分 28人</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>完成量 Top2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>深圳 23人</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>完成量 Top3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>海珠 20人</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>完成率 Bottom1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>佛山 44%</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>完成率 Bottom2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>汕头 48%</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>teng_long</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>完成率 Bottom3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>广分 80%</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>序时</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>目标退出率</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>绩差客户经理</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1-5月累计退出</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
         <v>44</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>目标 50%（96人）</t>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>完成率</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>46%</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>占绩差总人数</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>退出率 Top1-5</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>开发区/南沙/江门/汕头/梅州 100%</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>并列</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>退出人数 Top1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>深圳 8人</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>退出人数 Top2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>东莞 7人</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>退出人数 Top3</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>海珠 6人</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>退出率 Bottom1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>南京 20%</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>退出率 Bottom2</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>中山 20%</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>poor_perf</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>退出率 Bottom3</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>深圳 27%</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1-5月发生</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>15</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>已结案</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>11</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>胜诉</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>人（广州分行、信用卡中心）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>败诉</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>人（汕头分行、信用卡中心）</t>
         </is>
       </c>
     </row>
@@ -1638,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1666,265 +2859,442 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>headcount_total</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>中层总职数</t>
+          <t>中层干部总职数</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>211</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>headcount_filled</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>已配备</t>
+          <t>总行部门</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>194</v>
+        <v>100</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>headcount_vacancy</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>空缺</t>
+          <t>经营机构</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>111</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>市管领导干部</t>
+          <t>中层正职</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>高管人员</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>/</t>
+          <t>中层副职</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>157</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>人</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>派驻纪检监察组</t>
+          <t>已配备</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3</v>
+        <v>194</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>人（92%）</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>中层正职</t>
+          <t>尚空缺</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54</v>
-      </c>
-      <c r="D8" t="n">
-        <v>50</v>
-      </c>
-      <c r="E8" t="n">
-        <v>4</v>
+        <v>17</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>人（8%）</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>中层副职</t>
+          <t>总行已配备</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>157</v>
-      </c>
-      <c r="D9" t="n">
-        <v>144</v>
-      </c>
-      <c r="E9" t="n">
-        <v>13</v>
+        <v>93</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>人（空缺 7）</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>总行部门</t>
+          <t>经营已配备</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>100</v>
-      </c>
-      <c r="D10" t="n">
-        <v>93</v>
-      </c>
-      <c r="E10" t="n">
-        <v>7</v>
+        <v>101</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>人（空缺 10）</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>config_table</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>经营机构</t>
+          <t>正职已配备</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>111</v>
-      </c>
-      <c r="D11" t="n">
-        <v>101</v>
-      </c>
-      <c r="E11" t="n">
-        <v>10</v>
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>人（空缺 4）</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>adjustments</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>提拔</t>
+          <t>副职已配备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>人次</t>
+          <t>人（空缺 13）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>adjustments</t>
+          <t>position_table</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>降免职</t>
+          <t>市管领导干部</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>人次</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>高管人员</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>含工会主席、行长助理、首席风险官、首席信息官</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>派驻纪检监察组（不含组长）</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>中层正职</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>54</v>
+      </c>
+      <c r="D16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>副总级一把手 17 名</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>中层副职</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>157</v>
+      </c>
+      <c r="D17" t="n">
+        <v>144</v>
+      </c>
+      <c r="E17" t="n">
+        <v>13</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>副总 67 + 总助 74 + 经理 3，含 3 纪检</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>总行部门班子</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" t="n">
+        <v>93</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>position_table</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>经营机构班子</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>111</v>
+      </c>
+      <c r="D19" t="n">
+        <v>101</v>
+      </c>
+      <c r="E19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>含 3 纪检</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>adjustments</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>提拔</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>94</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>adjustments</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>降职、免职（含受处分）</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>14</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>adjustments</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>到龄转岗</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C22" t="n">
         <v>13</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>人次</t>
         </is>
@@ -1941,7 +3311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1969,7 +3339,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>salary_total</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1979,152 +3349,302 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15 亿元</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>亿元</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>salary_per_capita</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>人均薪酬</t>
+          <t>2025 年人均薪酬</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>24.3 万元</t>
+          <t>24.3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>含预发 2026 开门红 0.3 亿</t>
+          <t>万元（含预发 2026 开门红 0.3 亿）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pension_balance</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>企业年金余额</t>
+          <t>2026 年 1-5 月已发放</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17.44 亿元</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026.5</t>
+          <t>亿元</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tou_lang_count</t>
+          <t>pension</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>头狼评选</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>129</v>
+          <t>2025 年企业年金余额</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16.37</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026 Q1</t>
+          <t>亿元</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>monitoring</t>
+          <t>pension</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>监测人数</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>95</v>
+          <t>2026.5 余额</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>17.44</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>班子成员</t>
+          <t>亿元</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>monitoring</t>
+          <t>pension</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>监测人次</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>113</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>业绩监测</t>
-        </is>
-      </c>
+          <t>个人缴费比例</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>monitoring</t>
+          <t>pension</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>黑榜人数</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>督导函</t>
-        </is>
-      </c>
+          <t>单位缴费比例</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>pension</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025 补充医疗缴费</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7979</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pension</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>节余总额</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>亿元（含个人 + 单位住院）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pension</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026.5 节余</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>亿元（个人 1.6 + 单位 3002 万）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>监测人数</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>95</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>经营机构班子成员（不含到龄转岗及离职脱密期）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>监测人次</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>113</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>人 · 2026 Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>黑榜人数</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>人（首次触发监测督导）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>黑榜人次</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C15" t="n">
         <v>16</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>首次触发</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>人次 · 书面督导函</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>头狼评选</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>129</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>人 · 2026 Q1</t>
         </is>
       </c>
     </row>
@@ -2139,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2167,7 +3687,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>training_total</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2178,12 +3698,16 @@
       <c r="C2" t="n">
         <v>983</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>场</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>key_projects</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2194,223 +3718,435 @@
       <c r="C3" t="n">
         <v>55</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>exam_count</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>上岗资格人次</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1878</v>
+          <t>重点项目执行率</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>58.06%</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>35 场次</t>
+          <t>近期启动『走进华为 2.0』</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>key_projects_pct</t>
+          <t>key_projects</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>重点项目执行率</t>
+          <t>广银大讲堂</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.5806</v>
+        <v>5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>已完成 32/55</t>
+          <t>期</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>key_projects</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>董事会办公室</t>
+          <t>对公特训营</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>期</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>key_projects</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>私人银行部</t>
+          <t>个贷铁军培训</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>期</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>key_projects</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>金融同业部</t>
+          <t>办贷能力提升火线班</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>期</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>key_projects</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>金融市场部</t>
+          <t>校招新员工集中培训</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>100</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>期</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>战略客户部</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>100</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>董事会办公室</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>消保部</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>私人银行与财富管理部</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>机关纪委</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>100</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>金融同业部</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>安全保卫部</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>100</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>金融市场部</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>金融科技部</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>战略客户部</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>内控合规部</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>消费者权益保护部</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dept_execution</t>
+          <t>dept_top</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>机关纪委办公室</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dept_top</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>安全保卫部</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>dept_bottom</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>金融科技部</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>完成率</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>dept_bottom</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>内控合规部</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>完成率</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>dept_bottom</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>运营管理部</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14.29%</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>完成率</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>exam</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>上岗资格考试</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>35</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>场次</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>exam</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>参考人次</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1878</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>exam</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>涉及岗位</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>大岗位</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>